<commit_message>
feat(import): designation alias mapping for HR labels
The import script now accepts HR-system designation labels directly
in the XLSX without requiring users to look up system codes:
  DY CE / DY CE(GS)              -> DY_CE
  CAO / CAO/C / CAO(C)/RSP       -> CAO_C
  CE/Con (ROAD SAFETY PROJECT)   -> CE_C
  EXECUTIVE DIRECTOR/GATI SHAKTI(CIVIL-III) -> EDGS_CI

Alias resolution is logged in the Notes column of the output table.
Reference sheet in the template updated with the full alias mapping.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/user_import_template.xlsx
+++ b/scripts/user_import_template.xlsx
@@ -526,7 +526,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fill in the yellow columns (required). Grey columns are optional. Do not modify column headers.</t>
+          <t>Fill in the yellow columns (required). Grey columns are optional. Designation accepts both system codes (e.g. DY_CE) and HR labels (e.g. DY CE, CAO/C) -- see Reference sheet.</t>
         </is>
       </c>
     </row>
@@ -2196,7 +2196,7 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="C5:C204" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Designation" error="Choose a code from the dropdown or see the Reference sheet." type="list">
+    <dataValidation sqref="C5:C204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"EDGS_CI,CAO_C,CE_C,CE_PLANNING,DY_CE_C,DY_CE_PLANNING,DY_CE_DESIGN,DY_CE,SR_DEN,SR_DEN_CO,CBE,DY_CE_BRIDGE,CTE,DY_CE_TRACK,CPDE,PCE,DY_CSTE,SR_DSTE,CSTE_CON,CSTE_OL,PSCTE,DY_CEE,SR_DEE_TRD,CEE_CON,PCEE,SR_DOM,PCOM,SR_DCM,ADRM,DRM,CTPM,PCSO,CRS,GM,ADMIN,SUPER_ADMIN"</formula1>
     </dataValidation>
     <dataValidation sqref="D5:D204" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Zone" error="Choose a zone code from the dropdown or see the Reference sheet." type="list">
@@ -2213,7 +2213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2222,6 +2222,9 @@
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2242,6 +2245,13 @@
           <t>Field Notes</t>
         </is>
       </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>Designation Alias Mapping (HR labels accepted by import script)</t>
+        </is>
+      </c>
+      <c r="K1" s="8" t="n"/>
+      <c r="L1" s="8" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
@@ -2274,6 +2284,21 @@
           <t>Description</t>
         </is>
       </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>HR / External Label</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>System Code</t>
+        </is>
+      </c>
+      <c r="L2" s="9" t="inlineStr">
+        <is>
+          <t>System Label</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -2306,6 +2331,21 @@
           <t>Full name, e.g. 'Rajesh Kumar Singh'</t>
         </is>
       </c>
+      <c r="J3" s="10" t="inlineStr">
+        <is>
+          <t>DY CE</t>
+        </is>
+      </c>
+      <c r="K3" s="10" t="inlineStr">
+        <is>
+          <t>DY_CE</t>
+        </is>
+      </c>
+      <c r="L3" s="10" t="inlineStr">
+        <is>
+          <t>Dy CE</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -2338,6 +2378,21 @@
           <t>Official railnet email — must be unique</t>
         </is>
       </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>DY CE(GS)</t>
+        </is>
+      </c>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>DY_CE</t>
+        </is>
+      </c>
+      <c r="L4" s="10" t="inlineStr">
+        <is>
+          <t>Dy CE</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -2370,6 +2425,21 @@
           <t>Must match a code from the Designation Codes table</t>
         </is>
       </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>CAO/C</t>
+        </is>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>CAO_C</t>
+        </is>
+      </c>
+      <c r="L5" s="10" t="inlineStr">
+        <is>
+          <t>CAO/C</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -2402,6 +2472,21 @@
           <t>Leave blank for system/admin users (ADMIN, SUPER_ADMIN)</t>
         </is>
       </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>CAO</t>
+        </is>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>CAO_C</t>
+        </is>
+      </c>
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t>CAO/C</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -2434,6 +2519,21 @@
           <t>Optional HRMS / PF number. Leave blank if unknown.</t>
         </is>
       </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>CAO(C)/RSP</t>
+        </is>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>CAO_C</t>
+        </is>
+      </c>
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>CAO/C</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -2466,6 +2566,21 @@
           <t>Any free-text notes — not imported into the database</t>
         </is>
       </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>CE/C</t>
+        </is>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t>CE_C</t>
+        </is>
+      </c>
+      <c r="L8" s="10" t="inlineStr">
+        <is>
+          <t>CE/C</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -2488,6 +2603,21 @@
           <t>North Eastern Railway</t>
         </is>
       </c>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>CE/Con (ROAD SAFETY PROJECT)</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>CE_C</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>CE/C</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -2510,6 +2640,21 @@
           <t>Northeast Frontier Railway</t>
         </is>
       </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>EXECUTIVE DIRECTOR/GATI SHAKTI(CIVIL-III)</t>
+        </is>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>EDGS_CI</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>EDGS/C-I</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -2938,8 +3083,9 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="D1:E1"/>
+    <mergeCell ref="J1:L1"/>
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(zones): add Railway Board (RB) zone
V083 migration inserts RB zone for HQ/board-level users.
Updated user import template to include RB in the zone dropdown.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/user_import_template.xlsx
+++ b/scripts/user_import_template.xlsx
@@ -2200,7 +2200,7 @@
       <formula1>"EDGS_CI,CAO_C,CE_C,CE_PLANNING,DY_CE_C,DY_CE_PLANNING,DY_CE_DESIGN,DY_CE,SR_DEN,SR_DEN_CO,CBE,DY_CE_BRIDGE,CTE,DY_CE_TRACK,CPDE,PCE,DY_CSTE,SR_DSTE,CSTE_CON,CSTE_OL,PSCTE,DY_CEE,SR_DEE_TRD,CEE_CON,PCEE,SR_DOM,PCOM,SR_DCM,ADRM,DRM,CTPM,PCSO,CRS,GM,ADMIN,SUPER_ADMIN"</formula1>
     </dataValidation>
     <dataValidation sqref="D5:D204" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Zone" error="Choose a zone code from the dropdown or see the Reference sheet." type="list">
-      <formula1>"CR,ECR,ECOR,ER,KR,NCR,NER,NFR,NR,NWR,SCR,SECR,SER,SR,SWR,WCR,WR"</formula1>
+      <formula1>"CR,ECR,ECOR,ER,KR,NCR,NER,NFR,NR,NWR,SCR,SECR,SER,SR,SWR,WCR,WR,RB"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2865,6 +2865,16 @@
           <t>Sr DSTE</t>
         </is>
       </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>RB</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>Railway Board</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">

</xml_diff>